<commit_message>
docs(governanca): GRC, catálogo e qualidade de dados, STRIDE v2.0, dicionário, relatórios e notebook
</commit_message>
<xml_diff>
--- a/docs/stride/matriz-stride.xlsx
+++ b/docs/stride/matriz-stride.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U28"/>
+  <dimension ref="A1:U35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -650,12 +650,12 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>CNPJ ativo + natureza jurídica de associação/fundação; aprovação manual do Admin (regras 6.3); só ONG aprovada usa o caixa</t>
+          <t>Dígito verificador do CNPJ (inclusive alfanumérico) + consulta à Receita (situação ATIVA, natureza jurídica sem fins lucrativos) + aprovação manual do Admin (regras 6.3); só ONG aprovada usa o caixa</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Log de aprovação/reprovação; alerta de ONG com muitos aceites e poucas confirmações de entrega</t>
+          <t>Log de aprovação/reprovação; alerta de ONG com pedidos muito acima do que recebe (linha de base, regras 6.5/10.2)</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>Implementado (regra + dataset)</t>
+          <t>Implementado (v2.0)</t>
         </is>
       </c>
       <c r="Q2" s="2" t="n">
@@ -684,7 +684,7 @@
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>docs/regras-de-negocio.md §6.3; ongs.csv (3 pendentes, 2 reprovadas fora do matching); src/data/simulacao.py (ongs_ok)</t>
+          <t>src/validacao/documentos.py, receita.py; tests/validacao/test_receita.py; ongs.csv (3 pendentes, 2 reprovadas fora do matching)</t>
         </is>
       </c>
     </row>
@@ -881,12 +881,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>S5</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Integração com app de entrega</t>
+          <t>Consulta à Receita (BrasilAPI)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -896,17 +896,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Callback falso confirma uma entrega paga que não aconteceu</t>
+          <t>Resposta falsificada ou adulterada (DNS/MITM, serviço comprometido) faz um CNPJ inativo parecer ativo</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Webhook sem autenticação da origem</t>
+          <t>Confiar na resposta externa sem validar; aprovar por omissão quando o serviço cai</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Caixa solidário</t>
+          <t>Verificação de ONG</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>OWASP LLM05 (saída externa não confiável)</t>
         </is>
       </c>
       <c r="I5" s="2" t="n">
@@ -935,32 +935,32 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Webhook assinado (HMAC) e validado; a entrega só conta com confirmação da ONG</t>
+          <t>HTTPS sem seguir redirecionamento; resposta validada por esquema; CNPJ da resposta tem de ser o consultado; falha fechada (PENDENTE); aprovação humana final</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Conciliação diária: entregas pagas x eventos ENTREGA confirmados</t>
+          <t>Log de consultas PENDENTES e respostas fora do esquema</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>Estorno/contestação junto ao app e bloqueio do fluxo</t>
+          <t>Reconsulta e revisão manual</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>Planejado CP3</t>
+          <t>Implementado (v2.0)</t>
         </is>
       </c>
       <c r="Q5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="R5" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S5" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T5" s="6" t="inlineStr">
         <is>
@@ -969,44 +969,44 @@
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>regras §9 (livro-caixa com comprovante)</t>
+          <t>src/validacao/receita.py; tests/validacao/test_receita.py</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>S4</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Cadastro do lote</t>
+          <t>Integração com app de entrega</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>T - Tampering</t>
+          <t>S - Spoofing</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Doador informa validade falsa para passar na validade mínima (ex.: marmita vencida)</t>
+          <t>Callback falso confirma uma entrega paga que não aconteceu</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Confiar na validade digitada pelo doador</t>
+          <t>Webhook sem autenticação da origem</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Saúde de quem recebe</t>
+          <t>Caixa solidário</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Integridade / Segurança alimentar</t>
+          <t>Integridade</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1015,68 +1015,68 @@
         </is>
       </c>
       <c r="I6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="J6" s="2" t="n">
-        <v>5</v>
-      </c>
       <c r="K6" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
-          <t>Crítico</t>
+        <v>8</v>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>Médio</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Validade CALCULADA pelo sistema a partir de preparo + armazenamento (regras 4.2); validade mínima e rota expressa no código</t>
+          <t>Webhook assinado (HMAC) e validado; a entrega só conta com confirmação da ONG</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Inspeção da ONG na entrega (regras 6.2.1); reincidência por doador</t>
+          <t>Conciliação diária: entregas pagas x eventos ENTREGA confirmados</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>Suspensão do doador reincidente</t>
+          <t>Estorno/contestação junto ao app e bloqueio do fluxo</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>Implementado</t>
+          <t>Planejado CP3</t>
         </is>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R6" s="2" t="n">
         <v>4</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="T6" s="4" t="inlineStr">
-        <is>
-          <t>Médio</t>
+        <v>4</v>
+      </c>
+      <c r="T6" s="6" t="inlineStr">
+        <is>
+          <t>Baixo</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>src/regras/validade.py; tests/test_regras.py (4.2/4.3); RECUSA_INSPECAO em eventos.csv.gz</t>
+          <t>regras §9 (livro-caixa com comprovante)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Pipeline de treino</t>
+          <t>Cadastro do lote</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1086,92 +1086,92 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Envenenamento de dados: lotes falsos em massa para enviesar o Modelo 2 (ex.: fazer uma região parecer 'sempre salva')</t>
+          <t>Doador informa validade falsa para passar na validade mínima (ex.: marmita vencida)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Treinar com qualquer registro, sem confirmação do desfecho</t>
+          <t>Confiar na validade digitada pelo doador</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Modelos de IA, decisões de gasto</t>
+          <t>Saúde de quem recebe</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Integridade</t>
+          <t>Integridade / Segurança alimentar</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>OWASP LLM04 · MITRE ATLAS AML.T0020</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Validade CALCULADA pelo sistema a partir de preparo + armazenamento (regras 4.2); validade mínima e rota expressa no código; questionário obrigatório com declaração assinada (regras 4.5)</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Inspeção da ONG na entrega (regras 6.2.1); reincidência por doador; desvio do peso/volume do próprio histórico (10.2)</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>Suspensão do doador reincidente; a declaração assinada é a prova</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="n">
         <v>2</v>
-      </c>
-      <c r="J7" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="K7" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>Médio</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>Treino só com desfechos confirmados por duas partes (ONG + transportador); dataset versionado por SHA-256; revisão humana antes de promover modelo</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>Monitorar drift das features e da taxa de descarte por região</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>Rollback para a versão anterior do modelo (metadados versionados)</t>
-        </is>
-      </c>
-      <c r="P7" s="2" t="inlineStr">
-        <is>
-          <t>Parcial (hash do dataset e versão nos metadados)</t>
-        </is>
-      </c>
-      <c r="Q7" s="2" t="n">
-        <v>1</v>
       </c>
       <c r="R7" s="2" t="n">
         <v>4</v>
       </c>
       <c r="S7" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="T7" s="6" t="inlineStr">
-        <is>
-          <t>Baixo</t>
+        <v>8</v>
+      </c>
+      <c r="T7" s="4" t="inlineStr">
+        <is>
+          <t>Médio</t>
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>models/*.json (sha256_dataset, versão); src/models/treinar.py</t>
+          <t>src/regras/validade.py, questionario.py; tests/test_regras.py, test_questionario.py; RECUSA_INSPECAO e BLOQUEIO_QUESTIONARIO em eventos.csv.gz</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Artefatos de modelo (.joblib)</t>
+          <t>Pipeline de treino</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1181,92 +1181,92 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Arquivo do modelo substituído por um malicioso: executa código ao ser carregado (pickle)</t>
+          <t>Envenenamento de dados: lotes falsos em massa para enviesar o Modelo 2 (ex.: fazer uma região parecer 'sempre salva')</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Desserializar artefato sem verificar integridade</t>
+          <t>Treinar com qualquer registro, sem confirmação do desfecho</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Servidor da aplicação</t>
+          <t>Modelos de IA, decisões de gasto</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Integridade / Confidencialidade</t>
+          <t>Integridade</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>OWASP LLM03 · MITRE ATLAS AML.T0010</t>
+          <t>OWASP LLM04 · MITRE ATLAS AML.T0020</t>
         </is>
       </c>
       <c r="I8" s="2" t="n">
         <v>2</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="L8" s="5" t="inlineStr">
-        <is>
-          <t>Alto</t>
+        <v>8</v>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>Médio</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>SHA-256 do artefato gravado no treino e verificado antes do load; modelos fora do Git; imagem Docker imutável</t>
+          <t>Treino só com desfechos confirmados por duas partes (ONG + transportador); dataset versionado por SHA-256; qualidade de dados no pipeline; portão de promoção com teste fixo e aprovador diferente de quem treinou</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Falha de verificação gera alerta e bloqueia o start</t>
+          <t>Drift das entradas e saídas por PSI (10.2); checagens de qualidade de dados</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>Reimplantar a partir de artefato íntegro</t>
+          <t>Rollback para a versão anterior (RegistroDeVersoes)</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>Implementado</t>
+          <t>Implementado (v2.0)</t>
         </is>
       </c>
       <c r="Q8" s="2" t="n">
         <v>1</v>
       </c>
       <c r="R8" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="T8" s="4" t="inlineStr">
-        <is>
-          <t>Médio</t>
+        <v>4</v>
+      </c>
+      <c r="T8" s="6" t="inlineStr">
+        <is>
+          <t>Baixo</t>
         </is>
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>src/models/artefatos.py; tests/test_artefatos.py (artefato adulterado é recusado)</t>
+          <t>models/*.json (sha256_dataset); src/governanca/qualidade.py; src/observabilidade/drift.py; src/models/feedback.py (portão, rollback)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Cadeia de suprimentos (PyPI, Hugging Face, SEADE)</t>
+          <t>Artefatos de modelo (.joblib)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1276,22 +1276,22 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Dependência, modelo ou fonte de dados comprometidos/alterados na origem</t>
+          <t>Arquivo do modelo substituído por um malicioso: executa código ao ser carregado (pickle)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Versões flutuantes; baixar 'a última versão' sem conferência</t>
+          <t>Desserializar artefato sem verificar integridade</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Código, modelos, dados</t>
+          <t>Servidor da aplicação</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Integridade</t>
+          <t>Integridade / Confidencialidade</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1315,22 +1315,22 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>requirements com versões fixadas; modelos HF fixados por commit, só safetensors, trust_remote_code=False, licenças inventariadas (Apache-2.0, MIT); SHA-256 fixado da fonte IPVS</t>
+          <t>SHA-256 do artefato gravado no treino e verificado antes do load; modelos fora do Git; imagem Docker imutável</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Trivy/Dependabot no CI para CVEs; falha de hash interrompe a curadoria</t>
+          <t>Falha de verificação gera alerta e bloqueia o start</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>Fixar versão anterior íntegra; abrir incidente</t>
+          <t>Reimplantar a partir de artefato íntegro</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>Implementado (fixação e hashes); Trivy planejado CP2</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="Q9" s="2" t="n">
@@ -1349,19 +1349,19 @@
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>requirements.txt; src/models/nlp.py (REVISAO_EMBEDDINGS, REVISAO_NLI); src/data/curadoria_ipvs.py (SHA256_IPVS)</t>
+          <t>src/models/artefatos.py; tests/test_artefatos.py (artefato adulterado é recusado)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>T5</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Repositório / regras no código</t>
+          <t>Cadeia de suprimentos (PyPI, Hugging Face, SEADE)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1371,92 +1371,92 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Commit malicioso ou descuidado altera pesos do ranking, tetos do caixa ou validades</t>
+          <t>Dependência, modelo ou fonte de dados comprometidos/alterados na origem</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Push direto na main sem revisão nem testes</t>
+          <t>Versões flutuantes; baixar 'a última versão' sem conferência</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Regras de negócio</t>
+          <t>Código, modelos, dados</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Integridade / Governança</t>
+          <t>Integridade</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>OWASP LLM03 · MITRE ATLAS AML.T0010</t>
         </is>
       </c>
       <c r="I10" s="2" t="n">
         <v>2</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>Médio</t>
+        <v>10</v>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Branch protegida + PR com revisão; testes de regra obrigatórios no CI</t>
+          <t>requirements com versões fixadas; modelos HF fixados por commit, só safetensors, trust_remote_code=False, licenças inventariadas (Apache-2.0, MIT); SHA-256 fixado da fonte IPVS</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Histórico do Git; teste que falha denuncia a mudança</t>
+          <t>Trivy/Dependabot no CI para CVEs; falha de hash interrompe a curadoria</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>Reverter commit</t>
+          <t>Fixar versão anterior íntegra; abrir incidente</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>Parcial (60 testes); proteção de branch planejada CP2</t>
+          <t>Implementado (fixação e hashes); Trivy planejado CP2</t>
         </is>
       </c>
       <c r="Q10" s="2" t="n">
         <v>1</v>
       </c>
       <c r="R10" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="T10" s="6" t="inlineStr">
-        <is>
-          <t>Baixo</t>
+        <v>5</v>
+      </c>
+      <c r="T10" s="4" t="inlineStr">
+        <is>
+          <t>Médio</t>
         </is>
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>tests/test_regras.py</t>
+          <t>requirements.txt; src/models/nlp.py (REVISAO_EMBEDDINGS, REVISAO_NLI); src/data/curadoria_ipvs.py (SHA256_IPVS)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>T6</t>
+          <t>T5</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>KPIs de impacto</t>
+          <t>Repositório / regras no código</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1466,22 +1466,22 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Registros de entrega/kg inflados para maquiar o impacto (fraude de relatório social/ESG)</t>
+          <t>Commit malicioso ou descuidado altera pesos do ranking, tetos do caixa ou validades</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Entrega registrada por uma só parte; tabela editável</t>
+          <t>Push direto na main sem revisão nem testes</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Relatórios de impacto, reputação</t>
+          <t>Regras de negócio</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Integridade</t>
+          <t>Integridade / Governança</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1490,13 +1490,13 @@
         </is>
       </c>
       <c r="I11" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
@@ -1505,78 +1505,78 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Entrega confirmada por ONG e transportador; eventos append-only; RLS no Supabase</t>
+          <t>Branch protegida + PR com revisão; testes de regra obrigatórios no CI</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Conciliação kg doado x kg entregue por ONG</t>
+          <t>Histórico do Git; teste que falha denuncia a mudança</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>Correção dos KPIs e auditoria da ONG</t>
+          <t>Reverter commit</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>Parcial (trilha de eventos); append-only planejado CP3</t>
+          <t>Parcial (testes de regra e governança); proteção de branch planejada CP2</t>
         </is>
       </c>
       <c r="Q11" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R11" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S11" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="T11" s="4" t="inlineStr">
-        <is>
-          <t>Médio</t>
+        <v>4</v>
+      </c>
+      <c r="T11" s="6" t="inlineStr">
+        <is>
+          <t>Baixo</t>
         </is>
       </c>
       <c r="U11" s="2" t="inlineStr">
         <is>
-          <t>eventos.csv.gz</t>
+          <t>tests/test_regras.py</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>T6</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Trilha de auditoria</t>
+          <t>KPIs de impacto</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>R - Repudiation</t>
+          <t>T - Tampering</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>ONG nega ter aceitado/recebido um lote; gestor nega ter aprovado um gasto</t>
+          <t>Registros de entrega/kg inflados para maquiar o impacto (fraude de relatório social/ESG)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Ações sem registro de ator e horário</t>
+          <t>Entrega registrada por uma só parte; tabela editável</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Caixa, responsabilização</t>
+          <t>Relatórios de impacto, reputação</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Governança</t>
+          <t>Integridade</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1600,93 +1600,93 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Todo evento registra ator, ação, horário e detalhe (regras 10); aprovação explícita no caixa</t>
+          <t>Entrega confirmada por ONG e transportador; eventos append-only; RLS no Supabase</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Consulta à trilha por lote/ator</t>
+          <t>Conciliação kg doado x kg entregue por ONG</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>Resolução de disputa com a trilha como prova</t>
+          <t>Correção dos KPIs e auditoria da ONG</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>Implementado (formato e dataset)</t>
+          <t>Parcial (trilha de eventos); append-only planejado CP3</t>
         </is>
       </c>
       <c r="Q12" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R12" s="2" t="n">
         <v>3</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="T12" s="6" t="inlineStr">
-        <is>
-          <t>Baixo</t>
+        <v>6</v>
+      </c>
+      <c r="T12" s="4" t="inlineStr">
+        <is>
+          <t>Médio</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
-          <t>eventos.csv.gz (~245 mil eventos, 21 tipos); docs/dicionario-de-dados.md</t>
+          <t>eventos.csv.gz</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>T7</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Decisões da IA</t>
+          <t>Declaração de Doação</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>R - Repudiation</t>
+          <t>T - Tampering</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Não se consegue provar qual versão do modelo tomou uma decisão (ex.: acionou o pago)</t>
+          <t>Doador ou funcionário altera a declaração depois do fato (ex.: apagar que o alimento ficou exposto em buffet)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Modelo sem versionamento nem vínculo com os dados de treino</t>
+          <t>Documento editável, sem prova de integridade nem de origem</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Governança da IA</t>
+          <t>Responsabilidade sanitária e legal</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Governança</t>
+          <t>Integridade / Governança</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>NIST AI RMF (Medir) · ISO/IEC 42001</t>
+          <t>Lei 14.016/2020</t>
         </is>
       </c>
       <c r="I13" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
@@ -1695,22 +1695,22 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Metadados por modelo: versão, features, limiar, hash do dataset e do artefato; log com modelo + predição</t>
+          <t>JSON canônico + SHA-256 + assinatura RSA-PSS (3072 bits); repositório só de inclusão; correção = nova versão encadeada</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Relatório de métricas versionado</t>
+          <t>verificar / verificar_historico apontam conteúdo alterado ou versão quebrada</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>Reexecutar a decisão com a versão registrada</t>
+          <t>A versão original continua guardada e válida</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>Implementado</t>
+          <t>Implementado (v2.0)</t>
         </is>
       </c>
       <c r="Q13" s="2" t="n">
@@ -1729,59 +1729,59 @@
       </c>
       <c r="U13" s="2" t="inlineStr">
         <is>
-          <t>models/*.json; reports/metricas_modelos.json</t>
+          <t>src/seguranca/declaracao.py; tests/seguranca/test_declaracao.py</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>I1</t>
+          <t>T8</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Dados de doador PF</t>
+          <t>Trilha de auditoria (logs)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>I - Information Disclosure</t>
+          <t>T - Tampering</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Vazamento de CPF e endereço residencial de doadores pessoa física</t>
+          <t>Insider apaga ou edita linhas do log para esconder desvio no caixa ou aceite indevido</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Documento em claro; endereço exposto antes do match; hash sem segredo (quebrável por força bruta)</t>
+          <t>Log em arquivo comum, sem encadeamento; ou hash simples que o próprio insider recalcula</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Dados pessoais (LGPD)</t>
+          <t>Responsabilização</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Privacidade</t>
+          <t>Integridade</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>OWASP LLM02 · LGPD art. 46</t>
+          <t>MITRE ATT&amp;CK T1070 (Indicator Removal)</t>
         </is>
       </c>
       <c r="I14" s="2" t="n">
         <v>3</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
@@ -1790,32 +1790,32 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>HMAC-SHA256 com chave secreta; PF no centroide do setor; endereço só após o aceite; TLS e criptografia em repouso; retenção de 12 meses</t>
+          <t>Cadeia HMAC-SHA256 com chave fora do servidor de logs; âncora de retenção também selada</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>Auditoria de acesso a dados pessoais</t>
+          <t>verificar_cadeia aponta a linha exata</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>Plano de resposta a incidentes + comunicação à ANPD</t>
+          <t>Restaurar do backup e investigar quem tinha acesso de escrita</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>Parcial (minimização no dataset; HMAC na regra)</t>
+          <t>Implementado (v2.0)</t>
         </is>
       </c>
       <c r="Q14" s="2" t="n">
         <v>1</v>
       </c>
       <c r="R14" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T14" s="6" t="inlineStr">
         <is>
@@ -1824,49 +1824,49 @@
       </c>
       <c r="U14" s="2" t="inlineStr">
         <is>
-          <t>doadores.csv (sem documento em claro, PF no centroide); regras §11</t>
+          <t>src/observabilidade/registro.py; tests/observabilidade/test_registro.py (alteração, remoção, chave errada, âncora forjada)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>I2</t>
+          <t>T9</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Autorização por ONG</t>
+          <t>Feedback humano (RLHF adaptado)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>I - Information Disclosure</t>
+          <t>T - Tampering</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Uma ONG acessa lotes, endereços ou gastos de outra ONG (IDOR)</t>
+          <t>Atacante 'corrige' a IA em massa (ex.: marmita = não perecível) para envenenar o próximo modelo</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Autorização só no front-end ou feita pelo modelo</t>
+          <t>Usar toda correção como rótulo de treino</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Dados de lotes e parceiros</t>
+          <t>Modelos de IA</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Confidencialidade</t>
+          <t>Integridade</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>OWASP API1 (BOLA)</t>
+          <t>OWASP LLM04 · MITRE ATLAS AML.T0020</t>
         </is>
       </c>
       <c r="I15" s="2" t="n">
@@ -1885,32 +1885,32 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Row Level Security no Supabase por ONG; autorização na API (fora do modelo); testes de autorização</t>
+          <t>Só conta verificada; 20 correções/ator/dia; cota de 2% dos rótulos por ator; quarentena de ator com taxa de correção fora da linha de base; portão com teste fixo</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Log de acesso negado</t>
+          <t>Quarentena gera revisão humana</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>Correção da política e revisão dos acessos</t>
+          <t>Descartar o lote de feedback; rollback do modelo</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>Planejado CP3</t>
+          <t>Implementado (v2.0)</t>
         </is>
       </c>
       <c r="Q15" s="2" t="n">
         <v>1</v>
       </c>
       <c r="R15" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S15" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T15" s="6" t="inlineStr">
         <is>
@@ -1919,93 +1919,93 @@
       </c>
       <c r="U15" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>src/models/feedback.py; tests/models/test_feedback.py; reports/feedback_demo.json (NLP real: atacante em quarentena, 0 rótulos aceitos; sem a validação o veneno passaria no portão)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>I3</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>API de predição</t>
+          <t>Trilha de auditoria</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>I - Information Disclosure</t>
+          <t>R - Repudiation</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Consultas repetidas para copiar o Modelo 2 ou inferir dados de treino (extração/inversão)</t>
+          <t>ONG nega ter aceitado/recebido um lote; gestor nega ter aprovado um gasto</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>API aberta devolvendo probabilidades brutas</t>
+          <t>Ações sem registro de ator e horário</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Propriedade do modelo</t>
+          <t>Caixa, responsabilização</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Confidencialidade</t>
+          <t>Governança</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>MITRE ATLAS AML.T0024 / AML.T0040</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I16" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="L16" s="6" t="inlineStr">
-        <is>
-          <t>Baixo</t>
+        <v>9</v>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Médio</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Autenticação; rate limit; expor só a decisão (risco alto/baixo), não a probabilidade</t>
+          <t>Todo evento registra ator (pseudônimo), ação, horário, correlação e resultado (regras 10.1); trilha de auditoria encadeada por HMAC; declaração assinada por lote</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>Detecção de padrão de consulta anômalo</t>
+          <t>verificar_cadeia aponta linha alterada, apagada ou reordenada</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>Bloqueio do cliente</t>
+          <t>Resolução de disputa com a trilha e a declaração como prova</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>Planejado CP2</t>
+          <t>Implementado (v2.0)</t>
         </is>
       </c>
       <c r="Q16" s="2" t="n">
         <v>1</v>
       </c>
       <c r="R16" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S16" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T16" s="6" t="inlineStr">
         <is>
@@ -2014,114 +2014,114 @@
       </c>
       <c r="U16" s="2" t="inlineStr">
         <is>
-          <t>Modelo treinado com dados sintéticos, sem PII (impacto baixo)</t>
+          <t>src/observabilidade/registro.py; tests/observabilidade/test_registro.py; eventos.csv.gz</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>I4</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Segredos (Supabase, tokens)</t>
+          <t>Decisões da IA</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>I - Information Disclosure</t>
+          <t>R - Repudiation</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Chave service_role ou token vazados no repositório, nos logs ou no CI</t>
+          <t>Não se consegue provar qual versão do modelo tomou uma decisão (ex.: acionou o pago)</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Segredo em código ou em .env versionado</t>
+          <t>Modelo sem versionamento nem vínculo com os dados de treino</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Banco inteiro</t>
+          <t>Governança da IA</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Confidencialidade / Integridade</t>
+          <t>Governança</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NIST AI RMF (Medir) · ISO/IEC 42001</t>
         </is>
       </c>
       <c r="I17" s="2" t="n">
         <v>3</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="L17" s="5" t="inlineStr">
-        <is>
-          <t>Alto</t>
+        <v>9</v>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Médio</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>.gitignore bloqueia .env/.key/.pem; segredos no GitHub Secrets; service_role só no backend</t>
+          <t>Metadados por modelo: versão, features, limiar, hash do dataset e do artefato; TODA chamada de IA registrada (modelo, versão, entradas, saída, confiança, fallback)</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>Secret scanning (gitleaks/Trivy) no CI</t>
+          <t>Relatório de métricas versionado; taxa de fallback</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>Rotação imediata da chave vazada</t>
+          <t>Reexecutar a decisão com a versão registrada</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>Parcial (.gitignore); scanning planejado CP2</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="Q17" s="2" t="n">
         <v>1</v>
       </c>
       <c r="R17" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S17" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="T17" s="4" t="inlineStr">
-        <is>
-          <t>Médio</t>
+        <v>3</v>
+      </c>
+      <c r="T17" s="6" t="inlineStr">
+        <is>
+          <t>Baixo</t>
         </is>
       </c>
       <c r="U17" s="2" t="inlineStr">
         <is>
-          <t>.gitignore</t>
+          <t>models/*.json; src/models/controle.py; tests/models/test_controle.py</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>I5</t>
+          <t>I1</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Logs</t>
+          <t>Dados de doador PF</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -2131,17 +2131,17 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Logs guardam descrições livres e dados pessoais por tempo indeterminado</t>
+          <t>Vazamento de CPF e endereço residencial de doadores pessoa física</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Registrar tudo sem minimização nem retenção (caso AtendeMais, aula 6)</t>
+          <t>Documento em claro; endereço exposto antes do match; hash sem segredo (quebrável por força bruta)</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Dados pessoais</t>
+          <t>Dados pessoais (LGPD)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2151,51 +2151,51 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>OWASP LLM02</t>
+          <t>OWASP LLM02 · LGPD art. 46</t>
         </is>
       </c>
       <c r="I18" s="2" t="n">
         <v>3</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Médio</t>
+        <v>15</v>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Eventos com IDs pseudonimizados; texto livre não entra na trilha; retenção de 12 meses</t>
+          <t>HMAC-SHA256 com chave secreta; PF no centroide do setor; endereço só após o aceite; TLS e criptografia em repouso; retenção de 12 meses</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>Revisão periódica do conteúdo dos logs</t>
+          <t>Auditoria de acesso a dados pessoais</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>Expurgo e anonimização</t>
+          <t>Plano de resposta a incidentes + comunicação à ANPD</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>Implementado (formato da trilha)</t>
+          <t>Parcial (minimização no dataset; HMAC na regra)</t>
         </is>
       </c>
       <c r="Q18" s="2" t="n">
         <v>1</v>
       </c>
       <c r="R18" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S18" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T18" s="6" t="inlineStr">
         <is>
@@ -2204,19 +2204,19 @@
       </c>
       <c r="U18" s="2" t="inlineStr">
         <is>
-          <t>eventos.csv.gz (ator = ID, sem nomes nem texto livre)</t>
+          <t>doadores.csv (sem documento em claro, PF no centroide); regras §11</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>I6</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Mapa / localização de ONGs</t>
+          <t>Autorização por ONG</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -2226,17 +2226,17 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Exposição da localização de ONGs e de distribuições noturnas a pessoas mal-intencionadas</t>
+          <t>Uma ONG acessa lotes, endereços ou gastos de outra ONG (IDOR)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Mapa público com pontos exatos</t>
+          <t>Autorização só no front-end ou feita pelo modelo</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Segurança física de beneficiários e voluntários</t>
+          <t>Dados de lotes e parceiros</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -2246,41 +2246,41 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>OWASP API1 (BOLA)</t>
         </is>
       </c>
       <c r="I19" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>4</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Médio</t>
+        <v>12</v>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Mapa público só agregado por região (heatmap); localização exata só para quem tem match aceito</t>
+          <t>Row Level Security no Supabase por ONG; autorização na API (fora do modelo); testes de autorização</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>Revisão do que o dashboard público mostra</t>
+          <t>Log de acesso negado</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>Remover camada e revisar acessos</t>
+          <t>Correção da política e revisão dos acessos</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>Planejado CP3 (dashboard)</t>
+          <t>Planejado CP3</t>
         </is>
       </c>
       <c r="Q19" s="2" t="n">
@@ -2299,93 +2299,93 @@
       </c>
       <c r="U19" s="2" t="inlineStr">
         <is>
-          <t>regras §2.1 (índice por região)</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>I3</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Endpoint de NLP</t>
+          <t>API de predição</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>D - Denial of Service</t>
+          <t>I - Information Disclosure</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Entradas gigantes ou em massa esgotam a CPU e derrubam o free tier</t>
+          <t>Consultas repetidas para copiar o Modelo 2 ou inferir dados de treino (extração/inversão)</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Sem limite de tamanho nem de frequência</t>
+          <t>API aberta devolvendo probabilidades brutas</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Disponibilidade da plataforma</t>
+          <t>Propriedade do modelo</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Disponibilidade</t>
+          <t>Confidencialidade</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>OWASP LLM10 · MITRE ATLAS AML.T0029</t>
+          <t>MITRE ATLAS AML.T0024 / AML.T0040</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K20" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="J20" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="K20" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="L20" s="5" t="inlineStr">
-        <is>
-          <t>Alto</t>
+      <c r="L20" s="6" t="inlineStr">
+        <is>
+          <t>Baixo</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>Guardrail limita a 500 caracteres; classificador leve (4,6 ms/texto, antes 3,3 s com NLI); rate limit por usuário; timeout; formulário estruturado como alternativa</t>
+          <t>Autenticação; rate limit; expor só a decisão (risco alto/baixo), não a probabilidade</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>Monitorar latência e fila</t>
+          <t>Detecção de padrão de consulta anômalo</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>Degradar para o formulário sem NLP</t>
+          <t>Bloqueio do cliente</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>Parcial (limite de tamanho); rate limit planejado CP2</t>
+          <t>Planejado CP2</t>
         </is>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R20" s="2" t="n">
         <v>2</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T20" s="6" t="inlineStr">
         <is>
@@ -2394,44 +2394,44 @@
       </c>
       <c r="U20" s="2" t="inlineStr">
         <is>
-          <t>src/seguranca/guardrails.py; tests/seguranca/test_guardrails.py (entrada_gigante); reports/avaliacao_nlp.json (latência 3,3 s -&gt; 4,6 ms)</t>
+          <t>Modelo treinado com dados sintéticos, sem PII (impacto baixo)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>I4</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Cadastro de lotes</t>
+          <t>Segredos (Supabase, tokens)</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>D - Denial of Service</t>
+          <t>I - Information Disclosure</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Cadastro em massa de lotes falsos inunda as ONGs com ofertas (fadiga, recusas)</t>
+          <t>Chave service_role ou token vazados no repositório, nos logs ou no CI</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Sem limite por doador</t>
+          <t>Segredo em código ou em .env versionado</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Operação das ONGs</t>
+          <t>Banco inteiro</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Disponibilidade</t>
+          <t>Confidencialidade / Integridade</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -2443,200 +2443,200 @@
         <v>3</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>.gitignore bloqueia .env/.key/.pem; segredos no GitHub Secrets; service_role só no backend</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>Secret scanning (gitleaks/Trivy) no CI</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>Rotação imediata da chave vazada</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>Parcial (.gitignore); scanning planejado CP2</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R21" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S21" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="T21" s="4" t="inlineStr">
         <is>
           <t>Médio</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
-        <is>
-          <t>Rate limit por doador; doador verificado; reputação</t>
-        </is>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
-        <is>
-          <t>Alerta de volume anômalo por doador</t>
-        </is>
-      </c>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t>Suspender o doador e limpar as ofertas</t>
-        </is>
-      </c>
-      <c r="P21" s="2" t="inlineStr">
-        <is>
-          <t>Planejado CP2</t>
-        </is>
-      </c>
-      <c r="Q21" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="R21" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="S21" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="T21" s="6" t="inlineStr">
-        <is>
-          <t>Baixo</t>
-        </is>
-      </c>
       <c r="U21" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>.gitignore</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>I5</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Infraestrutura gratuita (Render/HF)</t>
+          <t>Logs</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>D - Denial of Service</t>
+          <t>I - Information Disclosure</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Serviço 'dorme' ou estoura a cota do free tier justamente num lote crítico</t>
+          <t>Logs guardam descrições livres e dados pessoais por tempo indeterminado</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Dependência de plano gratuito sem monitoramento</t>
+          <t>Registrar tudo sem minimização nem retenção (caso AtendeMais, aula 6)</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Disponibilidade, lotes críticos</t>
+          <t>Dados pessoais</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Disponibilidade</t>
+          <t>Privacidade</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>OWASP LLM02</t>
         </is>
       </c>
       <c r="I22" s="2" t="n">
         <v>3</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="L22" s="5" t="inlineStr">
-        <is>
-          <t>Alto</t>
+        <v>9</v>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Médio</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>Health check / keep-alive; alertas; a rota expressa cai para orientação de refrigeração</t>
+          <t>Log completo em COBERTURA e mínimo em CONTEÚDO: chaves proibidas removidas e CPF/CNPJ/e-mail/telefone mascarados no código; texto livre só como hash; retenção 90 dias (operacional) / 5 anos (auditoria)</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>Monitoramento de uptime</t>
+          <t>Teste que injeta dado pessoal e confere que não chega ao arquivo</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>Plano de contingência documentado</t>
+          <t>Expurgo por retenção (âncora selada mantém a cadeia)</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>Planejado CP3</t>
+          <t>Implementado (v2.0)</t>
         </is>
       </c>
       <c r="Q22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R22" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="R22" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="S22" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="T22" s="4" t="inlineStr">
-        <is>
-          <t>Médio</t>
+        <v>2</v>
+      </c>
+      <c r="T22" s="6" t="inlineStr">
+        <is>
+          <t>Baixo</t>
         </is>
       </c>
       <c r="U22" s="2" t="inlineStr">
         <is>
-          <t>regras §7.5 (orientação de refrigeração como fallback)</t>
+          <t>src/seguranca/minimizacao.py; src/observabilidade/registro.py; tests/observabilidade/test_registro.py</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>I6</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Caixa solidário</t>
+          <t>Mapa / localização de ONGs</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>D - Denial of Service</t>
+          <t>I - Information Disclosure</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Esgotamento do caixa por acionamentos pagos desnecessários ou abusivos</t>
+          <t>Exposição da localização de ONGs e de distribuições noturnas a pessoas mal-intencionadas</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Pagamento automático sem limites</t>
+          <t>Mapa público com pontos exatos</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Recursos do caixa</t>
+          <t>Segurança física de beneficiários e voluntários</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Disponibilidade / Governança</t>
+          <t>Confidencialidade</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>OWASP LLM06</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
@@ -2645,32 +2645,32 @@
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>Tetos de R$ 40 por entrega e R$ 200 por dia por ONG; gestor externo acima disso; pago só com espera estourada + risco alto</t>
+          <t>Mapa público só agregado por região (heatmap); localização exata só para quem tem match aceito</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>Relatório de gastos por ONG</t>
+          <t>Revisão do que o dashboard público mostra</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>Bloqueio preventivo do caixa da ONG</t>
+          <t>Remover camada e revisar acessos</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>Implementado</t>
+          <t>Planejado CP3 (dashboard)</t>
         </is>
       </c>
       <c r="Q23" s="2" t="n">
         <v>1</v>
       </c>
       <c r="R23" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S23" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T23" s="6" t="inlineStr">
         <is>
@@ -2679,90 +2679,90 @@
       </c>
       <c r="U23" s="2" t="inlineStr">
         <is>
-          <t>src/regras/logistica.py; tests/test_regras.py (caixa, pago)</t>
+          <t>regras §2.1 (índice por região)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>I7</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>NLP / texto livre</t>
+          <t>Mural de pedidos das ONGs</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>E - Elevation of Privilege</t>
+          <t>I - Information Disclosure</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Prompt injection no texto do doador para manipular a classificação ou 'dar ordens' ao sistema</t>
+          <t>Mural revela padrão de necessidade e localização de ONGs e de distribuições noturnas</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Tratar texto do usuário como instrução</t>
+          <t>Pedido publicado com endereço e horário</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Triagem, regras</t>
+          <t>Segurança de beneficiários e voluntários</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Integridade</t>
+          <t>Confidencialidade</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>OWASP LLM01 · MITRE ATLAS AML.T0051</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>3</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="L24" s="5" t="inlineStr">
-        <is>
-          <t>Alto</t>
+        <v>6</v>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Médio</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>Guardrail v2 (normalização + padrões); classificador só escolhe rótulo de lista FIXA (sem agência); doador confirma; regras revalidam</t>
+          <t>Mural agregado por região (categoria e kg), nunca com endereço; aviso só a doador que ativou, 1 por dia</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>Evento de bloqueio registrado para investigação</t>
+          <t>Revisão do que o mural expõe</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>Atualizar padrões a partir dos incidentes (reteste)</t>
+          <t>Remover pedido e revisar a exposição</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>Implementado</t>
+          <t>Regra definida (6.5); mural no CP3</t>
         </is>
       </c>
       <c r="Q24" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R24" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S24" s="2" t="n">
         <v>3</v>
@@ -2774,56 +2774,56 @@
       </c>
       <c r="U24" s="2" t="inlineStr">
         <is>
-          <t>reports/avaliacao_nlp.json: dataset 100% bloqueado; inéditos A 10/10 (após mitigação); B reservado 4/10 (risco residual aceito: impacto mínimo por arquitetura)</t>
+          <t>docs/regras-de-negocio.md §6.5</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Modelo 2 / cascata de transporte</t>
+          <t>Endpoint de NLP</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>E - Elevation of Privilege</t>
+          <t>D - Denial of Service</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>A IA passa a executar ações de impacto (pagar entregador) sem supervisão</t>
+          <t>Entradas gigantes ou em massa esgotam a CPU e derrubam o free tier</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Agência excessiva: saída do modelo vira ação</t>
+          <t>Sem limite de tamanho nem de frequência</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Caixa, confiança</t>
+          <t>Disponibilidade da plataforma</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Governança</t>
+          <t>Disponibilidade</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>OWASP LLM06 (Excessive Agency)</t>
+          <t>OWASP LLM10 · MITRE ATLAS AML.T0029</t>
         </is>
       </c>
       <c r="I25" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K25" s="2" t="n">
         <v>12</v>
@@ -2835,32 +2835,32 @@
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>A IA só recomenda; pago exige espera estourada + risco alto + tetos + confirmação da ONG ou do gestor</t>
+          <t>Guardrail limita a 500 caracteres; classificador leve (4,6 ms/texto, antes 3,3 s com NLI); limite de 120 req/min por chave + freio automático; formulário sem NLP como alternativa</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>Log de ACIONA_PAGO / APROVACAO_CAIXA</t>
+          <t>Linha de base de requisições e latência p95 (10.2)</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>Desligar a recomendação (voltar à heurística)</t>
+          <t>Desligar o NLP (o doador escolhe a categoria sozinho)</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>Implementado</t>
+          <t>Implementado (biblioteca; ligado na API no CP3)</t>
         </is>
       </c>
       <c r="Q25" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R25" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S25" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T25" s="6" t="inlineStr">
         <is>
@@ -2869,90 +2869,90 @@
       </c>
       <c r="U25" s="2" t="inlineStr">
         <is>
-          <t>src/regras/logistica.py (pode_acionar_pago, aprovacao_necessaria); tests/test_regras.py</t>
+          <t>src/seguranca/guardrails.py; tests/seguranca/test_guardrails.py (entrada_gigante); reports/avaliacao_nlp.json (latência 3,3 s -&gt; 4,6 ms)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Perfis e permissões (RBAC)</t>
+          <t>Cadastro de lotes</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>E - Elevation of Privilege</t>
+          <t>D - Denial of Service</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Usuário de ONG obtém papel de gestor/admin, ou gestor vinculado a uma ONG aprova o próprio gasto</t>
+          <t>Cadastro em massa de lotes falsos inunda as ONGs com ofertas (fadiga, recusas)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Papéis acumulados; checagem de permissão no cliente</t>
+          <t>Sem limite por doador</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Caixa, cadastro de ONGs</t>
+          <t>Operação das ONGs</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Integridade / Governança</t>
+          <t>Disponibilidade</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>OWASP API5 (BFLA)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I26" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J26" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K26" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>Limite de requisições; doador verificado (CNPJ/CPF); peso acima de 2 t vai para revisão humana</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>Alerta quando o volume do doador sai do PRÓPRIO histórico (mediana/MAD), antes de qualquer teto</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>Suspender o doador e limpar as ofertas</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>Implementado (v2.0)</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J26" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K26" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="L26" s="5" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="inlineStr">
-        <is>
-          <t>Um perfil por usuário; segregação de funções (quem pede não aprova; admin não aprova caixa); RBAC no backend + RLS</t>
-        </is>
-      </c>
-      <c r="N26" s="2" t="inlineStr">
-        <is>
-          <t>Alerta de mudança de papel</t>
-        </is>
-      </c>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>Revogar o papel e revisar as aprovações</t>
-        </is>
-      </c>
-      <c r="P26" s="2" t="inlineStr">
-        <is>
-          <t>Parcial (regra definida); RBAC planejado CP3</t>
-        </is>
-      </c>
-      <c r="Q26" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="R26" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S26" s="2" t="n">
         <v>4</v>
@@ -2964,195 +2964,860 @@
       </c>
       <c r="U26" s="2" t="inlineStr">
         <is>
-          <t>regras §3 e §9</t>
+          <t>src/observabilidade/anomalias.py; tests/observabilidade/test_anomalias.py; src/regras/cadastro.py</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>E4</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Saída do classificador</t>
+          <t>Infraestrutura gratuita (Render/HF)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>E - Elevation of Privilege</t>
+          <t>D - Denial of Service</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>A saída do modelo é gravada/usada por outro componente sem validação</t>
+          <t>Serviço 'dorme' ou estoura a cota do free tier justamente num lote crítico</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Confiar na saída da IA como dado válido</t>
+          <t>Dependência de plano gratuito sem monitoramento</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Integridade dos lotes</t>
+          <t>Disponibilidade, lotes críticos</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Integridade</t>
+          <t>Disponibilidade</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>OWASP LLM05 (Improper Output Handling)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I27" s="2" t="n">
         <v>3</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="L27" s="4" t="inlineStr">
+        <v>12</v>
+      </c>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>Health check / keep-alive; alertas; a rota expressa cai para orientação de refrigeração</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>Monitoramento de uptime</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>Plano de contingência documentado</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>Planejado CP3</t>
+        </is>
+      </c>
+      <c r="Q27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="R27" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="S27" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="T27" s="4" t="inlineStr">
         <is>
           <t>Médio</t>
         </is>
       </c>
-      <c r="M27" s="2" t="inlineStr">
-        <is>
-          <t>Sugestão nunca gravada sem confirmação; valores restritos a enums fechados; regras revalidam depois</t>
-        </is>
-      </c>
-      <c r="N27" s="2" t="inlineStr">
-        <is>
-          <t>Divergência sugestão x confirmação monitorada</t>
-        </is>
-      </c>
-      <c r="O27" s="2" t="inlineStr">
-        <is>
-          <t>Corrigir o registro</t>
-        </is>
-      </c>
-      <c r="P27" s="2" t="inlineStr">
-        <is>
-          <t>Implementado</t>
-        </is>
-      </c>
-      <c r="Q27" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R27" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="S27" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="T27" s="6" t="inlineStr">
-        <is>
-          <t>Baixo</t>
-        </is>
-      </c>
       <c r="U27" s="2" t="inlineStr">
         <is>
-          <t>src/models/nlp.py (requer_confirmacao); src/regras/dominio.py (enums)</t>
+          <t>regras §7.5 (orientação de refrigeração como fallback)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>E5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>CI/CD (GitHub Actions)</t>
+          <t>Caixa solidário</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>E - Elevation of Privilege</t>
+          <t>D - Denial of Service</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Action de terceiro maliciosa ou workflow com permissão ampla publica código malicioso</t>
+          <t>Esgotamento do caixa por acionamentos pagos desnecessários ou abusivos</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Actions por tag flutuante; token do workflow com escrita total</t>
+          <t>Pagamento automático sem limites</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Produção</t>
+          <t>Recursos do caixa</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Integridade</t>
+          <t>Disponibilidade / Governança</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>MITRE ATT&amp;CK T1195 (Supply Chain Compromise)</t>
+          <t>OWASP LLM06</t>
         </is>
       </c>
       <c r="I28" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="L28" s="5" t="inlineStr">
-        <is>
-          <t>Alto</t>
+        <v>9</v>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Médio</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>Actions fixadas por SHA; permissions mínimas; segredos em ambiente protegido; Bandit/Trivy como security gate</t>
+          <t>Tetos de R$ 40 por entrega e R$ 200 por dia por ONG; gestor externo acima disso; pago só com espera estourada + risco alto</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>Log de execuções do pipeline</t>
+          <t>Relatório de gastos por ONG</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>Revogar tokens e reimplantar</t>
+          <t>Bloqueio preventivo do caixa da ONG</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>Planejado CP2</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="Q28" s="2" t="n">
         <v>1</v>
       </c>
       <c r="R28" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="S28" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="T28" s="6" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+      <c r="U28" s="2" t="inlineStr">
+        <is>
+          <t>src/regras/logistica.py; tests/test_regras.py (caixa, pago)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Observabilidade / freio automático</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>D - Denial of Service</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Atacante provoca o freio sobre um usuário legítimo (ou enche o painel de alertas para esconder um ataque real)</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Bloqueio automático permanente; alerta a cada evento</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Disponibilidade, atenção da equipe</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Disponibilidade</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J29" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K29" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>Freio só para sinais de segurança, reversível em 15 min e revisado por humano; sinal de negócio nunca bloqueia; alerta só quando o nível sobe na janela</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>Freios aplicados ficam na trilha de auditoria</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>Admin libera o freio</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>Implementado (v2.0)</t>
+        </is>
+      </c>
+      <c r="Q29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R29" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="S29" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="T29" s="6" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+      <c r="U29" s="2" t="inlineStr">
+        <is>
+          <t>src/observabilidade/freio.py, anomalias.py; tests/observabilidade/test_anomalias.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>NLP / texto livre</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>E - Elevation of Privilege</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Prompt injection no texto do doador para manipular a classificação ou 'dar ordens' ao sistema</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Tratar texto do usuário como instrução</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Triagem, regras</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Integridade</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>OWASP LLM01 · MITRE ATLAS AML.T0051</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="S28" s="2" t="n">
+      <c r="J30" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K30" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>Guardrail v2 (normalização + padrões); classificador só escolhe rótulo de lista FIXA (sem agência); doador confirma; regras revalidam</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>Evento de bloqueio registrado para investigação</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>Atualizar padrões a partir dos incidentes (reteste)</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="Q30" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="R30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S30" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="T30" s="6" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>reports/avaliacao_nlp.json: dataset 100% bloqueado; inéditos A 10/10 (após mitigação); B reservado 4/10 (risco residual aceito: impacto mínimo por arquitetura)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Modelo 2 / cascata de transporte</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>E - Elevation of Privilege</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>A IA passa a executar ações de impacto (pagar entregador) sem supervisão</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Agência excessiva: saída do modelo vira ação</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Caixa, confiança</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Governança</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>OWASP LLM06 (Excessive Agency)</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J31" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="T28" s="6" t="inlineStr">
+      <c r="K31" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="L31" s="5" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>A IA só recomenda (agência zero); pago exige espera estourada + risco alto + tetos + confirmação da ONG ou do gestor</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>Log de cada predição e de ACIONA_PAGO / APROVACAO_CAIXA; caixa avisa ao passar de 70% e 90% do teto</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>Desligar o modelo por interruptor auditado (volta à heurística)</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="Q31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R31" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="S31" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="T31" s="6" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="U28" s="2" t="inlineStr">
+      <c r="U31" s="2" t="inlineStr">
+        <is>
+          <t>src/regras/logistica.py; src/models/controle.py (Interruptores); docs/governanca/analise-agencia-ia.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Perfis e permissões (RBAC)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>E - Elevation of Privilege</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Usuário de ONG obtém papel de gestor/admin, ou gestor vinculado a uma ONG aprova o próprio gasto</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Papéis acumulados; checagem de permissão no cliente</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Caixa, cadastro de ONGs</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Integridade / Governança</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>OWASP API5 (BFLA)</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J32" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="L32" s="5" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>Um perfil por usuário; segregação de funções (quem pede não aprova; admin não aprova caixa); RBAC no backend + RLS</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>Alerta de mudança de papel</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>Revogar o papel e revisar as aprovações</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>Parcial (regra definida); RBAC planejado CP3</t>
+        </is>
+      </c>
+      <c r="Q32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R32" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="S32" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="T32" s="6" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+      <c r="U32" s="2" t="inlineStr">
+        <is>
+          <t>regras §3 e §9</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>E4</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Saída do classificador</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>E - Elevation of Privilege</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>A saída do modelo é gravada/usada por outro componente sem validação</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Confiar na saída da IA como dado válido</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Integridade dos lotes</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Integridade</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>OWASP LLM05 (Improper Output Handling)</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J33" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K33" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>Sugestão nunca gravada sem confirmação; saída validada contra lista fechada e [0, 1] na camada de controle; piso de segurança no M1</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>Divergência sugestão x confirmação monitorada (vira feedback auditado)</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>Fallback automático para a regra</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="Q33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R33" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="S33" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="T33" s="6" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+      <c r="U33" s="2" t="inlineStr">
+        <is>
+          <t>src/models/controle.py; tests/models/test_controle.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>E6</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Validação de entrada (atribuição em massa)</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>E - Elevation of Privilege</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Cliente envia campos extras ou tipos trocados ("aprovado": true, "prioridade": "CRITICA", "peso": "1e9") para pular regras</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Esquema permissivo que aceita campo desconhecido e converte tipos em silêncio</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Regras de negócio</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Integridade</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>OWASP API3 (BOPLA)</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J34" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="K34" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>Esquemas com extra=forbid e strict; listas fechadas; faixas; datas com fuso; coerência entre campos; a prioridade nunca vem do cliente</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>Validação rejeitada vai para o log operacional (campo e regra, sem o valor)</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>Bloqueio pelo freio se houver rajada</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>Implementado (v2.0)</t>
+        </is>
+      </c>
+      <c r="Q34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R34" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="S34" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="T34" s="6" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+      <c r="U34" s="2" t="inlineStr">
+        <is>
+          <t>src/validacao/esquemas.py; tests/validacao/test_esquemas.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>E5</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>CI/CD (GitHub Actions)</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>E - Elevation of Privilege</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Action de terceiro maliciosa ou workflow com permissão ampla publica código malicioso</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Actions por tag flutuante; token do workflow com escrita total</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Produção</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Integridade</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>MITRE ATT&amp;CK T1195 (Supply Chain Compromise)</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J35" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K35" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="L35" s="5" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>Actions fixadas por SHA; permissions mínimas; segredos em ambiente protegido; Bandit/Trivy como security gate</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>Log de execuções do pipeline</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>Revogar tokens e reimplantar</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>Planejado CP2</t>
+        </is>
+      </c>
+      <c r="Q35" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R35" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="S35" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="T35" s="6" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+      <c r="U35" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3169,7 +3834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3277,6 +3942,60 @@
       <c r="E4" t="inlineStr">
         <is>
           <t>IA só recomenda; justificativa visível; humano decide ações de impacto (aula 7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Eficiência logística x comida perdida</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>A preferência por pares complementares (busca x entrega) pode levar o lote a uma ONG mais distante</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Ética / Operacional</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Complementaridade multiplicada pelo acesso (custo medido: ~0,2 p.p. de descarte); monitorar descarte por complementaridade</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Fadiga de alertas</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Muitos alertas fazem a equipe ignorar o que importa</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Três níveis; alerta só quando o nível sobe na janela; aquecimento antes de alertar; sinais de negócio não bloqueiam</t>
         </is>
       </c>
     </row>
@@ -3318,7 +4037,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -3331,7 +4050,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -3344,7 +4063,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C4" t="n">
         <v>9</v>
@@ -3360,7 +4079,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>